<commit_message>
fix: desktop app - notification dedup, bigger click targets, button hover-glow styles
</commit_message>
<xml_diff>
--- a/PROJECT_LOG.xlsx
+++ b/PROJECT_LOG.xlsx
@@ -787,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1438,6 +1438,262 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fix checkbox GestureDetector conflict - checkbox toggles not blocked by parent onTap</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>home_screen.dart</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Fix backup screen Windows path separator handling</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>backup_screen.dart</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Fix recurring todo reminder cancellation and rescheduling</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>todo_provider.dart</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Fix pomodoro stats to query real DB minutes instead of local count</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>database_helper.dart, stats_screen.dart</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Wrap WidgetService.updateWidget() in try-catch to prevent crash</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>todo_provider.dart, pomodoro_provider.dart</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>feat</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Apply consistent button styling globally (padding 8x28, radius 20, font 14/600)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>app_theme.dart</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Fix speech_to_text plugin to v7.4.0, core library desugaring for Android build</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>pubspec.yaml, android/app/build.gradle.kts</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Build APK (60.8 MB) and push to GitHub release v3.1.0</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>(build artifacts)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: remove floating timer, add Document PiP pop-out ticker
</commit_message>
<xml_diff>
--- a/PROJECT_LOG.xlsx
+++ b/PROJECT_LOG.xlsx
@@ -787,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1694,6 +1694,38 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>3.1.1+2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Desktop app v1.4.0-1.5.0 - timer removal, PiP pop out ticker</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>src/index.html, src/styles.css, src/app.js, package.json</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>opencode</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>